<commit_message>
M3-普通塔同步：Normal 接入分等级 prefab（Tower_Normal0|1|2 与 mkii/mkiii 美术）
四层同步（复用 Power/Retard 已确立的分等级模式）：
- 配置：TowerInfo.xlsx id 1/2/3 resName Tower_Normal → Tower_Normal0/1/2；
  另 Pierce/Laser 占位行(id 10~15)同步指向 Tower_Normal0；重导 Luban（== succ ==）
- 寻址：ResTable 单条 Tower_Normal 拆为 Tower_Normal0/1/2（Normal/ 目录）+ 补 mkii/mkiii 贴图登记
- 代码：GameFlowManager 预载加 Normal0/1/2；BaseTower/TowerPlacement 兜底字面量同步；
  TowerPrefabConverter 清单扩 9 项 + TowerPath 加 Normal 分支 + Specs 三档
- 资源：新增 Normal/ 三个 prefab（AB=tower_normal）与四级美术；删旧 Tower_Normal.prefab

校验：9 个 resName 全有 ResTable 登记且路径存在；三 prefab 引 NormalTower GUID、节点结构一致；
五项静态检查全 PASS。设计文档 §Z.12；记忆已更新（塔分等级口径）
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/TowerInfo.xlsx
+++ b/Luban/Config/Datas/TowerInfo.xlsx
@@ -1474,7 +1474,7 @@
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal0</t>
         </is>
       </c>
       <c r="F4" s="0" t="n">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal1</t>
         </is>
       </c>
       <c r="F5" s="0" t="n">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal2</t>
         </is>
       </c>
       <c r="F6" s="0" t="n">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal0</t>
         </is>
       </c>
       <c r="F21" s="0" t="n">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal0</t>
         </is>
       </c>
       <c r="F22" s="0" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal0</t>
         </is>
       </c>
       <c r="F23" s="0" t="n">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal0</t>
         </is>
       </c>
       <c r="F24" s="0" t="n">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal0</t>
         </is>
       </c>
       <c r="F25" s="0" t="n">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Tower_Normal</t>
+          <t>Tower_Normal0</t>
         </is>
       </c>
       <c r="F26" s="0" t="n">

</xml_diff>